<commit_message>
Mark more systems to avoid sampling for now
</commit_message>
<xml_diff>
--- a/data/Milliman_et_al_2014_WIYN_single_lined_orbits.xlsx
+++ b/data/Milliman_et_al_2014_WIYN_single_lined_orbits.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="104">
   <si>
     <t xml:space="preserve">#</t>
   </si>
@@ -329,6 +329,9 @@
   </si>
   <si>
     <t xml:space="preserve">stampede</t>
+  </si>
+  <si>
+    <t xml:space="preserve">check if solved</t>
   </si>
 </sst>
 </file>
@@ -494,7 +497,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="21">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -555,15 +558,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -576,14 +571,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1277,7 +1264,6 @@
       <c r="A79" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="B79" s="15"/>
       <c r="C79" s="0" t="n">
         <v>49002</v>
       </c>
@@ -1326,10 +1312,10 @@
       <c r="R79" s="0" t="n">
         <v>0.03</v>
       </c>
-      <c r="S79" s="16" t="n">
+      <c r="S79" s="15" t="n">
         <v>0.0259</v>
       </c>
-      <c r="T79" s="16" t="n">
+      <c r="T79" s="15" t="n">
         <v>0.0017</v>
       </c>
       <c r="U79" s="0" t="n">
@@ -1339,73 +1325,71 @@
         <v>20</v>
       </c>
     </row>
-    <row r="80" s="18" customFormat="true" ht="16" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="15"/>
-      <c r="B80" s="17"/>
-      <c r="C80" s="18" t="n">
+    <row r="80" s="16" customFormat="true" ht="16" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="0"/>
+      <c r="C80" s="16" t="n">
         <v>14008</v>
       </c>
-      <c r="D80" s="18" t="n">
+      <c r="D80" s="16" t="n">
         <v>1.71953</v>
       </c>
-      <c r="E80" s="18" t="n">
+      <c r="E80" s="16" t="n">
         <v>2.4E-005</v>
       </c>
-      <c r="F80" s="18" t="n">
+      <c r="F80" s="16" t="n">
         <v>860</v>
       </c>
-      <c r="G80" s="18" t="n">
+      <c r="G80" s="16" t="n">
         <v>2.6</v>
       </c>
-      <c r="H80" s="18" t="n">
+      <c r="H80" s="16" t="n">
         <v>0.9</v>
       </c>
-      <c r="I80" s="18" t="n">
+      <c r="I80" s="16" t="n">
         <v>45.3</v>
       </c>
-      <c r="J80" s="18" t="n">
+      <c r="J80" s="16" t="n">
         <v>1.3</v>
       </c>
-      <c r="K80" s="19" t="n">
+      <c r="K80" s="17" t="n">
         <v>0.02</v>
       </c>
-      <c r="L80" s="18" t="n">
+      <c r="L80" s="16" t="n">
         <v>0.03</v>
       </c>
-      <c r="M80" s="18" t="n">
+      <c r="M80" s="16" t="n">
         <v>300</v>
       </c>
-      <c r="N80" s="18" t="n">
+      <c r="N80" s="16" t="n">
         <v>80</v>
       </c>
-      <c r="O80" s="18" t="n">
+      <c r="O80" s="16" t="n">
         <v>52959.5</v>
       </c>
-      <c r="P80" s="18" t="n">
+      <c r="P80" s="16" t="n">
         <v>0.4</v>
       </c>
-      <c r="Q80" s="18" t="n">
+      <c r="Q80" s="16" t="n">
         <v>1.07</v>
       </c>
-      <c r="R80" s="18" t="n">
+      <c r="R80" s="16" t="n">
         <v>0.03</v>
       </c>
-      <c r="S80" s="20" t="n">
+      <c r="S80" s="18" t="n">
         <v>0.0166</v>
       </c>
-      <c r="T80" s="20" t="n">
+      <c r="T80" s="18" t="n">
         <v>0.0015</v>
       </c>
-      <c r="U80" s="18" t="n">
+      <c r="U80" s="16" t="n">
         <v>2.93</v>
       </c>
-      <c r="V80" s="18" t="n">
+      <c r="V80" s="16" t="n">
         <v>14</v>
       </c>
     </row>
     <row r="81" s="8" customFormat="true" ht="16" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="15"/>
-      <c r="B81" s="21"/>
+      <c r="A81" s="0"/>
       <c r="C81" s="8" t="n">
         <v>32006</v>
       </c>
@@ -1471,7 +1455,6 @@
       <c r="A82" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="B82" s="15"/>
       <c r="C82" s="0" t="n">
         <v>66004</v>
       </c>
@@ -1520,10 +1503,10 @@
       <c r="R82" s="0" t="n">
         <v>0.023</v>
       </c>
-      <c r="S82" s="16" t="n">
+      <c r="S82" s="15" t="n">
         <v>0.0135</v>
       </c>
-      <c r="T82" s="16" t="n">
+      <c r="T82" s="15" t="n">
         <v>0.0008</v>
       </c>
       <c r="U82" s="0" t="n">
@@ -1537,7 +1520,9 @@
       <c r="A83" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="B83" s="15"/>
+      <c r="B83" s="0" t="s">
+        <v>103</v>
+      </c>
       <c r="C83" s="0" t="n">
         <v>13001</v>
       </c>
@@ -1586,10 +1571,10 @@
       <c r="R83" s="0" t="n">
         <v>0.06</v>
       </c>
-      <c r="S83" s="16" t="n">
+      <c r="S83" s="15" t="n">
         <v>0.073</v>
       </c>
-      <c r="T83" s="16" t="n">
+      <c r="T83" s="15" t="n">
         <v>0.004</v>
       </c>
       <c r="U83" s="0" t="n">
@@ -1599,67 +1584,67 @@
         <v>16</v>
       </c>
     </row>
-    <row r="84" s="18" customFormat="true" ht="16" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="15"/>
-      <c r="B84" s="15"/>
-      <c r="C84" s="18" t="n">
+    <row r="84" s="16" customFormat="true" ht="16" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="0"/>
+      <c r="B84" s="0"/>
+      <c r="C84" s="16" t="n">
         <v>35025</v>
       </c>
-      <c r="D84" s="18" t="n">
+      <c r="D84" s="16" t="n">
         <v>4.64123</v>
       </c>
-      <c r="E84" s="18" t="n">
+      <c r="E84" s="16" t="n">
         <v>0.00013</v>
       </c>
-      <c r="F84" s="18" t="n">
+      <c r="F84" s="16" t="n">
         <v>199.4</v>
       </c>
-      <c r="G84" s="18" t="n">
+      <c r="G84" s="16" t="n">
         <v>2.45</v>
       </c>
-      <c r="H84" s="18" t="n">
+      <c r="H84" s="16" t="n">
         <v>0.22</v>
       </c>
-      <c r="I84" s="18" t="n">
+      <c r="I84" s="16" t="n">
         <v>39.2</v>
       </c>
-      <c r="J84" s="18" t="n">
+      <c r="J84" s="16" t="n">
         <v>0.5</v>
       </c>
-      <c r="K84" s="19" t="n">
+      <c r="K84" s="17" t="n">
         <v>0.208</v>
       </c>
-      <c r="L84" s="18" t="n">
+      <c r="L84" s="16" t="n">
         <v>0.012</v>
       </c>
-      <c r="M84" s="18" t="n">
+      <c r="M84" s="16" t="n">
         <v>117.2</v>
       </c>
-      <c r="N84" s="18" t="n">
+      <c r="N84" s="16" t="n">
         <v>2.4</v>
       </c>
-      <c r="O84" s="18" t="n">
+      <c r="O84" s="16" t="n">
         <v>51999.66</v>
       </c>
-      <c r="P84" s="18" t="n">
+      <c r="P84" s="16" t="n">
         <v>0.03</v>
       </c>
-      <c r="Q84" s="18" t="n">
+      <c r="Q84" s="16" t="n">
         <v>2.45</v>
       </c>
-      <c r="R84" s="18" t="n">
+      <c r="R84" s="16" t="n">
         <v>0.03</v>
       </c>
-      <c r="S84" s="20" t="n">
+      <c r="S84" s="18" t="n">
         <v>0.0271</v>
       </c>
-      <c r="T84" s="20" t="n">
+      <c r="T84" s="18" t="n">
         <v>0.001</v>
       </c>
-      <c r="U84" s="18" t="n">
+      <c r="U84" s="16" t="n">
         <v>0.74</v>
       </c>
-      <c r="V84" s="18" t="n">
+      <c r="V84" s="16" t="n">
         <v>17</v>
       </c>
     </row>
@@ -1667,7 +1652,6 @@
       <c r="A85" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="B85" s="15"/>
       <c r="C85" s="0" t="n">
         <v>60006</v>
       </c>
@@ -1716,10 +1700,10 @@
       <c r="R85" s="0" t="n">
         <v>0.024</v>
       </c>
-      <c r="S85" s="16" t="n">
+      <c r="S85" s="15" t="n">
         <v>0.0296</v>
       </c>
-      <c r="T85" s="16" t="n">
+      <c r="T85" s="15" t="n">
         <v>0.0006</v>
       </c>
       <c r="U85" s="0" t="n">
@@ -1733,7 +1717,6 @@
       <c r="A86" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="B86" s="15"/>
       <c r="C86" s="0" t="n">
         <v>57004</v>
       </c>
@@ -1782,10 +1765,10 @@
       <c r="R86" s="0" t="n">
         <v>0.03</v>
       </c>
-      <c r="S86" s="16" t="n">
+      <c r="S86" s="15" t="n">
         <v>0.0595</v>
       </c>
-      <c r="T86" s="16" t="n">
+      <c r="T86" s="15" t="n">
         <v>0.001</v>
       </c>
       <c r="U86" s="0" t="n">
@@ -1796,7 +1779,6 @@
       </c>
     </row>
     <row r="87" s="8" customFormat="true" ht="16" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="21"/>
       <c r="C87" s="8" t="n">
         <v>33002</v>
       </c>
@@ -1821,7 +1803,7 @@
       <c r="J87" s="8" t="n">
         <v>0.5</v>
       </c>
-      <c r="K87" s="21" t="n">
+      <c r="K87" s="8" t="n">
         <v>0.022</v>
       </c>
       <c r="L87" s="8" t="n">
@@ -1858,75 +1840,72 @@
         <v>18</v>
       </c>
     </row>
-    <row r="88" s="23" customFormat="true" ht="16" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="88" s="19" customFormat="true" ht="16" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="B88" s="22"/>
-      <c r="C88" s="23" t="n">
+      <c r="C88" s="19" t="n">
         <v>46013</v>
       </c>
-      <c r="D88" s="23" t="n">
+      <c r="D88" s="19" t="n">
         <v>14.2111</v>
       </c>
-      <c r="E88" s="23" t="n">
+      <c r="E88" s="19" t="n">
         <v>0.0015</v>
       </c>
-      <c r="F88" s="23" t="n">
+      <c r="F88" s="19" t="n">
         <v>105.4</v>
       </c>
-      <c r="G88" s="23" t="n">
+      <c r="G88" s="19" t="n">
         <v>2.3</v>
       </c>
-      <c r="H88" s="23" t="n">
+      <c r="H88" s="19" t="n">
         <v>0.3</v>
       </c>
-      <c r="I88" s="23" t="n">
+      <c r="I88" s="19" t="n">
         <v>10.8</v>
       </c>
-      <c r="J88" s="23" t="n">
+      <c r="J88" s="19" t="n">
         <v>0.5</v>
       </c>
-      <c r="K88" s="24" t="n">
+      <c r="K88" s="20" t="n">
         <v>0.53</v>
       </c>
-      <c r="L88" s="23" t="n">
+      <c r="L88" s="19" t="n">
         <v>0.04</v>
       </c>
-      <c r="M88" s="23" t="n">
+      <c r="M88" s="19" t="n">
         <v>256</v>
       </c>
-      <c r="N88" s="23" t="n">
+      <c r="N88" s="19" t="n">
         <v>5</v>
       </c>
-      <c r="O88" s="23" t="n">
+      <c r="O88" s="19" t="n">
         <v>51878.89</v>
       </c>
-      <c r="P88" s="23" t="n">
+      <c r="P88" s="19" t="n">
         <v>0.11</v>
       </c>
-      <c r="Q88" s="23" t="n">
+      <c r="Q88" s="19" t="n">
         <v>1.79</v>
       </c>
-      <c r="R88" s="23" t="n">
+      <c r="R88" s="19" t="n">
         <v>0.1</v>
       </c>
-      <c r="S88" s="23" t="n">
+      <c r="S88" s="19" t="n">
         <v>0.00113</v>
       </c>
-      <c r="T88" s="23" t="n">
+      <c r="T88" s="19" t="n">
         <v>0.00018</v>
       </c>
-      <c r="U88" s="23" t="n">
+      <c r="U88" s="19" t="n">
         <v>1.41</v>
       </c>
-      <c r="V88" s="23" t="n">
+      <c r="V88" s="19" t="n">
         <v>26</v>
       </c>
     </row>
     <row r="89" s="8" customFormat="true" ht="16" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A89" s="21"/>
-      <c r="B89" s="21"/>
       <c r="C89" s="8" t="n">
         <v>3002</v>
       </c>
@@ -1951,7 +1930,7 @@
       <c r="J89" s="8" t="n">
         <v>0.5</v>
       </c>
-      <c r="K89" s="21" t="n">
+      <c r="K89" s="8" t="n">
         <v>0.022</v>
       </c>
       <c r="L89" s="8" t="n">
@@ -1988,7 +1967,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="90" s="23" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="90" s="19" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="8" t="s">
         <v>102</v>
       </c>
@@ -2058,7 +2037,6 @@
       <c r="A91" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="B91" s="15"/>
       <c r="C91" s="0" t="n">
         <v>59003</v>
       </c>
@@ -2107,10 +2085,10 @@
       <c r="R91" s="0" t="n">
         <v>0.11</v>
       </c>
-      <c r="S91" s="16" t="n">
+      <c r="S91" s="15" t="n">
         <v>0.0622</v>
       </c>
-      <c r="T91" s="16" t="n">
+      <c r="T91" s="15" t="n">
         <v>0.0022</v>
       </c>
       <c r="U91" s="0" t="n">
@@ -2120,7 +2098,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="92" s="23" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="92" s="19" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="8" t="s">
         <v>102</v>
       </c>
@@ -2186,7 +2164,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="93" s="23" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="93" s="19" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="8" t="s">
         <v>102</v>
       </c>
@@ -2252,74 +2230,72 @@
         <v>15</v>
       </c>
     </row>
-    <row r="94" s="23" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="94" s="19" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="B94" s="22"/>
-      <c r="C94" s="23" t="n">
+      <c r="C94" s="19" t="n">
         <v>35020</v>
       </c>
-      <c r="D94" s="23" t="n">
+      <c r="D94" s="19" t="n">
         <v>24.737</v>
       </c>
-      <c r="E94" s="23" t="n">
+      <c r="E94" s="19" t="n">
         <v>0.005</v>
       </c>
-      <c r="F94" s="23" t="n">
+      <c r="F94" s="19" t="n">
         <v>45.4</v>
       </c>
-      <c r="G94" s="23" t="n">
+      <c r="G94" s="19" t="n">
         <v>1.4</v>
       </c>
-      <c r="H94" s="23" t="n">
+      <c r="H94" s="19" t="n">
         <v>0.17</v>
       </c>
-      <c r="I94" s="23" t="n">
+      <c r="I94" s="19" t="n">
         <v>12.4</v>
       </c>
-      <c r="J94" s="23" t="n">
+      <c r="J94" s="19" t="n">
         <v>0.5</v>
       </c>
-      <c r="K94" s="24" t="n">
+      <c r="K94" s="20" t="n">
         <v>0.36</v>
       </c>
-      <c r="L94" s="23" t="n">
+      <c r="L94" s="19" t="n">
         <v>0.03</v>
       </c>
-      <c r="M94" s="23" t="n">
+      <c r="M94" s="19" t="n">
         <v>136</v>
       </c>
-      <c r="N94" s="23" t="n">
+      <c r="N94" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="O94" s="23" t="n">
+      <c r="O94" s="19" t="n">
         <v>52042.16</v>
       </c>
-      <c r="P94" s="23" t="n">
+      <c r="P94" s="19" t="n">
         <v>0.19</v>
       </c>
-      <c r="Q94" s="23" t="n">
+      <c r="Q94" s="19" t="n">
         <v>3.93</v>
       </c>
-      <c r="R94" s="23" t="n">
+      <c r="R94" s="19" t="n">
         <v>0.15</v>
       </c>
-      <c r="S94" s="23" t="n">
+      <c r="S94" s="19" t="n">
         <v>0.004</v>
       </c>
-      <c r="T94" s="23" t="n">
+      <c r="T94" s="19" t="n">
         <v>0.0004</v>
       </c>
-      <c r="U94" s="23" t="n">
+      <c r="U94" s="19" t="n">
         <v>0.58</v>
       </c>
-      <c r="V94" s="23" t="n">
+      <c r="V94" s="19" t="n">
         <v>15</v>
       </c>
     </row>
     <row r="95" s="8" customFormat="true" ht="16" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A95" s="21"/>
       <c r="C95" s="8" t="n">
         <v>24012</v>
       </c>
@@ -2344,7 +2320,7 @@
       <c r="J95" s="8" t="n">
         <v>0.3</v>
       </c>
-      <c r="K95" s="21" t="n">
+      <c r="K95" s="8" t="n">
         <v>0.004</v>
       </c>
       <c r="L95" s="8" t="n">
@@ -2382,7 +2358,6 @@
       </c>
     </row>
     <row r="96" s="8" customFormat="true" ht="16" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A96" s="21"/>
       <c r="C96" s="8" t="n">
         <v>39013</v>
       </c>
@@ -2407,7 +2382,7 @@
       <c r="J96" s="8" t="n">
         <v>0.8</v>
       </c>
-      <c r="K96" s="21" t="n">
+      <c r="K96" s="8" t="n">
         <v>0.06</v>
       </c>
       <c r="L96" s="8" t="n">
@@ -2562,10 +2537,10 @@
       <c r="R98" s="0" t="n">
         <v>0.6</v>
       </c>
-      <c r="S98" s="16" t="n">
+      <c r="S98" s="15" t="n">
         <v>0.0005</v>
       </c>
-      <c r="T98" s="16" t="n">
+      <c r="T98" s="15" t="n">
         <v>0.0003</v>
       </c>
       <c r="U98" s="0" t="n">
@@ -2693,10 +2668,10 @@
       <c r="R100" s="0" t="n">
         <v>1.5</v>
       </c>
-      <c r="S100" s="16" t="n">
+      <c r="S100" s="15" t="n">
         <v>0.013</v>
       </c>
-      <c r="T100" s="16" t="n">
+      <c r="T100" s="15" t="n">
         <v>0.006</v>
       </c>
       <c r="U100" s="0" t="n">
@@ -2758,10 +2733,10 @@
       <c r="R101" s="0" t="n">
         <v>0.3</v>
       </c>
-      <c r="S101" s="16" t="n">
+      <c r="S101" s="15" t="n">
         <v>0.0451</v>
       </c>
-      <c r="T101" s="16" t="n">
+      <c r="T101" s="15" t="n">
         <v>0.0022</v>
       </c>
       <c r="U101" s="0" t="n">
@@ -3021,10 +2996,10 @@
       <c r="R105" s="0" t="n">
         <v>0.4</v>
       </c>
-      <c r="S105" s="16" t="n">
+      <c r="S105" s="15" t="n">
         <v>0.0425</v>
       </c>
-      <c r="T105" s="16" t="n">
+      <c r="T105" s="15" t="n">
         <v>0.0022</v>
       </c>
       <c r="U105" s="0" t="n">
@@ -3347,10 +3322,10 @@
       <c r="R110" s="0" t="n">
         <v>0.4</v>
       </c>
-      <c r="S110" s="16" t="n">
+      <c r="S110" s="15" t="n">
         <v>0.058</v>
       </c>
-      <c r="T110" s="16" t="n">
+      <c r="T110" s="15" t="n">
         <v>0.003</v>
       </c>
       <c r="U110" s="0" t="n">
@@ -3409,10 +3384,10 @@
       <c r="R111" s="0" t="n">
         <v>0.4</v>
       </c>
-      <c r="S111" s="16" t="n">
+      <c r="S111" s="15" t="n">
         <v>0.0336</v>
       </c>
-      <c r="T111" s="16" t="n">
+      <c r="T111" s="15" t="n">
         <v>0.0017</v>
       </c>
       <c r="U111" s="0" t="n">
@@ -3471,10 +3446,10 @@
       <c r="R112" s="0" t="n">
         <v>0.5</v>
       </c>
-      <c r="S112" s="16" t="n">
+      <c r="S112" s="15" t="n">
         <v>0.0135</v>
       </c>
-      <c r="T112" s="16" t="n">
+      <c r="T112" s="15" t="n">
         <v>0.0012</v>
       </c>
       <c r="U112" s="0" t="n">
@@ -3533,10 +3508,10 @@
       <c r="R113" s="0" t="n">
         <v>2.3</v>
       </c>
-      <c r="S113" s="16" t="n">
+      <c r="S113" s="15" t="n">
         <v>0.0033</v>
       </c>
-      <c r="T113" s="16" t="n">
+      <c r="T113" s="15" t="n">
         <v>0.0019</v>
       </c>
       <c r="U113" s="0" t="n">
@@ -3595,10 +3570,10 @@
       <c r="R114" s="0" t="n">
         <v>0.3</v>
       </c>
-      <c r="S114" s="16" t="n">
+      <c r="S114" s="15" t="n">
         <v>0.00138</v>
       </c>
-      <c r="T114" s="16" t="n">
+      <c r="T114" s="15" t="n">
         <v>0.00015</v>
       </c>
       <c r="U114" s="0" t="n">
@@ -3657,10 +3632,10 @@
       <c r="R115" s="0" t="n">
         <v>1.6</v>
       </c>
-      <c r="S115" s="16" t="n">
+      <c r="S115" s="15" t="n">
         <v>0.026</v>
       </c>
-      <c r="T115" s="16" t="n">
+      <c r="T115" s="15" t="n">
         <v>0.004</v>
       </c>
       <c r="U115" s="0" t="n">
@@ -3719,10 +3694,10 @@
       <c r="R116" s="0" t="n">
         <v>1.4</v>
       </c>
-      <c r="S116" s="16" t="n">
+      <c r="S116" s="15" t="n">
         <v>0.0015</v>
       </c>
-      <c r="T116" s="16" t="n">
+      <c r="T116" s="15" t="n">
         <v>0.0006</v>
       </c>
       <c r="U116" s="0" t="n">
@@ -3781,10 +3756,10 @@
       <c r="R117" s="0" t="n">
         <v>14</v>
       </c>
-      <c r="S117" s="16" t="n">
+      <c r="S117" s="15" t="n">
         <v>0.0077</v>
       </c>
-      <c r="T117" s="16" t="n">
+      <c r="T117" s="15" t="n">
         <v>0.014</v>
       </c>
       <c r="U117" s="0" t="n">
@@ -3843,10 +3818,10 @@
       <c r="R118" s="0" t="n">
         <v>0.8</v>
       </c>
-      <c r="S118" s="16" t="n">
+      <c r="S118" s="15" t="n">
         <v>0.1</v>
       </c>
-      <c r="T118" s="16" t="n">
+      <c r="T118" s="15" t="n">
         <v>0.005</v>
       </c>
       <c r="U118" s="0" t="n">
@@ -3905,10 +3880,10 @@
       <c r="R119" s="0" t="n">
         <v>0.8</v>
       </c>
-      <c r="S119" s="16" t="n">
+      <c r="S119" s="15" t="n">
         <v>0.071</v>
       </c>
-      <c r="T119" s="16" t="n">
+      <c r="T119" s="15" t="n">
         <v>0.004</v>
       </c>
       <c r="U119" s="0" t="n">
@@ -3967,10 +3942,10 @@
       <c r="R120" s="0" t="n">
         <v>0.8</v>
       </c>
-      <c r="S120" s="16" t="n">
+      <c r="S120" s="15" t="n">
         <v>0.0017</v>
       </c>
-      <c r="T120" s="16" t="n">
+      <c r="T120" s="15" t="n">
         <v>0.0003</v>
       </c>
       <c r="U120" s="0" t="n">
@@ -4029,10 +4004,10 @@
       <c r="R121" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="S121" s="16" t="n">
+      <c r="S121" s="15" t="n">
         <v>0.009</v>
       </c>
-      <c r="T121" s="16" t="n">
+      <c r="T121" s="15" t="n">
         <v>0.003</v>
       </c>
       <c r="U121" s="0" t="n">
@@ -4091,10 +4066,10 @@
       <c r="R122" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="S122" s="16" t="n">
+      <c r="S122" s="15" t="n">
         <v>0.079</v>
       </c>
-      <c r="T122" s="16" t="n">
+      <c r="T122" s="15" t="n">
         <v>0.013</v>
       </c>
       <c r="U122" s="0" t="n">
@@ -4153,10 +4128,10 @@
       <c r="R123" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="S123" s="16" t="n">
+      <c r="S123" s="15" t="n">
         <v>0.0083</v>
       </c>
-      <c r="T123" s="16" t="n">
+      <c r="T123" s="15" t="n">
         <v>0.0016</v>
       </c>
       <c r="U123" s="0" t="n">
@@ -4215,10 +4190,10 @@
       <c r="R124" s="0" t="n">
         <v>9</v>
       </c>
-      <c r="S124" s="16" t="n">
+      <c r="S124" s="15" t="n">
         <v>0.034</v>
       </c>
-      <c r="T124" s="16" t="n">
+      <c r="T124" s="15" t="n">
         <v>0.015</v>
       </c>
       <c r="U124" s="0" t="n">
@@ -4277,10 +4252,10 @@
       <c r="R125" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="S125" s="16" t="n">
+      <c r="S125" s="15" t="n">
         <v>0.015</v>
       </c>
-      <c r="T125" s="16" t="n">
+      <c r="T125" s="15" t="n">
         <v>0.003</v>
       </c>
       <c r="U125" s="0" t="n">
@@ -4339,10 +4314,10 @@
       <c r="R126" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="S126" s="16" t="n">
+      <c r="S126" s="15" t="n">
         <v>0.00017</v>
       </c>
-      <c r="T126" s="16" t="n">
+      <c r="T126" s="15" t="n">
         <v>0.00012</v>
       </c>
       <c r="U126" s="0" t="n">
@@ -4401,10 +4376,10 @@
       <c r="R127" s="0" t="n">
         <v>1.3</v>
       </c>
-      <c r="S127" s="16" t="n">
+      <c r="S127" s="15" t="n">
         <v>0.0349</v>
       </c>
-      <c r="T127" s="16" t="n">
+      <c r="T127" s="15" t="n">
         <v>0.0019</v>
       </c>
       <c r="U127" s="0" t="n">
@@ -4463,10 +4438,10 @@
       <c r="R128" s="0" t="n">
         <v>2.1</v>
       </c>
-      <c r="S128" s="16" t="n">
+      <c r="S128" s="15" t="n">
         <v>0.0082</v>
       </c>
-      <c r="T128" s="16" t="n">
+      <c r="T128" s="15" t="n">
         <v>0.0012</v>
       </c>
       <c r="U128" s="0" t="n">
@@ -4525,10 +4500,10 @@
       <c r="R129" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="S129" s="16" t="n">
+      <c r="S129" s="15" t="n">
         <v>0.025</v>
       </c>
-      <c r="T129" s="16" t="n">
+      <c r="T129" s="15" t="n">
         <v>0.003</v>
       </c>
       <c r="U129" s="0" t="n">
@@ -4587,10 +4562,10 @@
       <c r="R130" s="0" t="n">
         <v>40</v>
       </c>
-      <c r="S130" s="16" t="n">
+      <c r="S130" s="15" t="n">
         <v>0.11</v>
       </c>
-      <c r="T130" s="16" t="n">
+      <c r="T130" s="15" t="n">
         <v>0.12</v>
       </c>
       <c r="U130" s="0" t="n">
@@ -4649,10 +4624,10 @@
       <c r="R131" s="0" t="n">
         <v>50</v>
       </c>
-      <c r="S131" s="16" t="n">
+      <c r="S131" s="15" t="n">
         <v>10.9</v>
       </c>
-      <c r="T131" s="16" t="n">
+      <c r="T131" s="15" t="n">
         <v>0.011</v>
       </c>
       <c r="U131" s="0" t="n">
@@ -4711,10 +4686,10 @@
       <c r="R132" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="S132" s="16" t="n">
+      <c r="S132" s="15" t="n">
         <v>0.621</v>
       </c>
-      <c r="T132" s="16" t="n">
+      <c r="T132" s="15" t="n">
         <v>0.02</v>
       </c>
       <c r="U132" s="0" t="n">
@@ -4773,10 +4748,10 @@
       <c r="R133" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="S133" s="16" t="n">
+      <c r="S133" s="15" t="n">
         <v>0.027</v>
       </c>
-      <c r="T133" s="16" t="n">
+      <c r="T133" s="15" t="n">
         <v>0.006</v>
       </c>
       <c r="U133" s="0" t="n">
@@ -4835,10 +4810,10 @@
       <c r="R134" s="0" t="n">
         <v>2.1</v>
       </c>
-      <c r="S134" s="16" t="n">
+      <c r="S134" s="15" t="n">
         <v>0.0241</v>
       </c>
-      <c r="T134" s="16" t="n">
+      <c r="T134" s="15" t="n">
         <v>0.0021</v>
       </c>
       <c r="U134" s="0" t="n">
@@ -4897,10 +4872,10 @@
       <c r="R135" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="S135" s="16" t="n">
+      <c r="S135" s="15" t="n">
         <v>0.66</v>
       </c>
-      <c r="T135" s="16" t="n">
+      <c r="T135" s="15" t="n">
         <v>0.08</v>
       </c>
       <c r="U135" s="0" t="n">
@@ -4959,10 +4934,10 @@
       <c r="R136" s="0" t="n">
         <v>9</v>
       </c>
-      <c r="S136" s="16" t="n">
+      <c r="S136" s="15" t="n">
         <v>0.026</v>
       </c>
-      <c r="T136" s="16" t="n">
+      <c r="T136" s="15" t="n">
         <v>0.007</v>
       </c>
       <c r="U136" s="0" t="n">
@@ -5021,10 +4996,10 @@
       <c r="R137" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="S137" s="16" t="n">
+      <c r="S137" s="15" t="n">
         <v>0.0066</v>
       </c>
-      <c r="T137" s="16" t="n">
+      <c r="T137" s="15" t="n">
         <v>0.0018</v>
       </c>
       <c r="U137" s="0" t="n">
@@ -5083,10 +5058,10 @@
       <c r="R138" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="S138" s="16" t="n">
+      <c r="S138" s="15" t="n">
         <v>0.0172</v>
       </c>
-      <c r="T138" s="16" t="n">
+      <c r="T138" s="15" t="n">
         <v>0.0025</v>
       </c>
       <c r="U138" s="0" t="n">
@@ -5145,10 +5120,10 @@
       <c r="R139" s="0" t="n">
         <v>17</v>
       </c>
-      <c r="S139" s="16" t="n">
+      <c r="S139" s="15" t="n">
         <v>0.003</v>
       </c>
-      <c r="T139" s="16" t="n">
+      <c r="T139" s="15" t="n">
         <v>0.003</v>
       </c>
       <c r="U139" s="0" t="n">
@@ -5207,10 +5182,10 @@
       <c r="R140" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="S140" s="16" t="n">
+      <c r="S140" s="15" t="n">
         <v>0.0201</v>
       </c>
-      <c r="T140" s="16" t="n">
+      <c r="T140" s="15" t="n">
         <v>0.0015</v>
       </c>
       <c r="U140" s="0" t="n">
@@ -5269,10 +5244,10 @@
       <c r="R141" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="S141" s="16" t="n">
+      <c r="S141" s="15" t="n">
         <v>0.0225</v>
       </c>
-      <c r="T141" s="16" t="n">
+      <c r="T141" s="15" t="n">
         <v>0.0022</v>
       </c>
       <c r="U141" s="0" t="n">
@@ -5331,10 +5306,10 @@
       <c r="R142" s="0" t="n">
         <v>9</v>
       </c>
-      <c r="S142" s="16" t="n">
+      <c r="S142" s="15" t="n">
         <v>0.0066</v>
       </c>
-      <c r="T142" s="16" t="n">
+      <c r="T142" s="15" t="n">
         <v>0.0022</v>
       </c>
       <c r="U142" s="0" t="n">
@@ -5393,10 +5368,10 @@
       <c r="R143" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="S143" s="16" t="n">
+      <c r="S143" s="15" t="n">
         <v>0.0079</v>
       </c>
-      <c r="T143" s="16" t="n">
+      <c r="T143" s="15" t="n">
         <v>0.0015</v>
       </c>
       <c r="U143" s="0" t="n">
@@ -5455,10 +5430,10 @@
       <c r="R144" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="S144" s="16" t="n">
+      <c r="S144" s="15" t="n">
         <v>0.015</v>
       </c>
-      <c r="T144" s="16" t="n">
+      <c r="T144" s="15" t="n">
         <v>0.004</v>
       </c>
       <c r="U144" s="0" t="n">
@@ -5517,10 +5492,10 @@
       <c r="R145" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="S145" s="16" t="n">
+      <c r="S145" s="15" t="n">
         <v>0.0098</v>
       </c>
-      <c r="T145" s="16" t="n">
+      <c r="T145" s="15" t="n">
         <v>0.0016</v>
       </c>
       <c r="U145" s="0" t="n">
@@ -5579,10 +5554,10 @@
       <c r="R146" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="S146" s="16" t="n">
+      <c r="S146" s="15" t="n">
         <v>0.043</v>
       </c>
-      <c r="T146" s="16" t="n">
+      <c r="T146" s="15" t="n">
         <v>0.004</v>
       </c>
       <c r="U146" s="0" t="n">
@@ -5641,10 +5616,10 @@
       <c r="R147" s="0" t="n">
         <v>12</v>
       </c>
-      <c r="S147" s="16" t="n">
+      <c r="S147" s="15" t="n">
         <v>0.022</v>
       </c>
-      <c r="T147" s="16" t="n">
+      <c r="T147" s="15" t="n">
         <v>0.005</v>
       </c>
       <c r="U147" s="0" t="n">
@@ -5703,10 +5678,10 @@
       <c r="R148" s="0" t="n">
         <v>19</v>
       </c>
-      <c r="S148" s="16" t="n">
+      <c r="S148" s="15" t="n">
         <v>0.106</v>
       </c>
-      <c r="T148" s="16" t="n">
+      <c r="T148" s="15" t="n">
         <v>0.022</v>
       </c>
       <c r="U148" s="0" t="n">
@@ -5765,10 +5740,10 @@
       <c r="R149" s="0" t="n">
         <v>110</v>
       </c>
-      <c r="S149" s="16" t="n">
+      <c r="S149" s="15" t="n">
         <v>0.2</v>
       </c>
-      <c r="T149" s="16" t="n">
+      <c r="T149" s="15" t="n">
         <v>0.19</v>
       </c>
       <c r="U149" s="0" t="n">
@@ -5827,10 +5802,10 @@
       <c r="R150" s="0" t="n">
         <v>8</v>
       </c>
-      <c r="S150" s="16" t="n">
+      <c r="S150" s="15" t="n">
         <v>0.051</v>
       </c>
-      <c r="T150" s="16" t="n">
+      <c r="T150" s="15" t="n">
         <v>0.005</v>
       </c>
       <c r="U150" s="0" t="n">
@@ -5889,10 +5864,10 @@
       <c r="R151" s="0" t="n">
         <v>23</v>
       </c>
-      <c r="S151" s="16" t="n">
+      <c r="S151" s="15" t="n">
         <v>0.012</v>
       </c>
-      <c r="T151" s="16" t="n">
+      <c r="T151" s="15" t="n">
         <v>0.005</v>
       </c>
       <c r="U151" s="0" t="n">
@@ -5951,10 +5926,10 @@
       <c r="R152" s="0" t="n">
         <v>12</v>
       </c>
-      <c r="S152" s="16" t="n">
+      <c r="S152" s="15" t="n">
         <v>0.011</v>
       </c>
-      <c r="T152" s="16" t="n">
+      <c r="T152" s="15" t="n">
         <v>0.003</v>
       </c>
       <c r="U152" s="0" t="n">
@@ -6013,10 +5988,10 @@
       <c r="R153" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="S153" s="16" t="n">
+      <c r="S153" s="15" t="n">
         <v>0.022</v>
       </c>
-      <c r="T153" s="16" t="n">
+      <c r="T153" s="15" t="n">
         <v>0.003</v>
       </c>
       <c r="U153" s="0" t="n">
@@ -6075,10 +6050,10 @@
       <c r="R154" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="S154" s="16" t="n">
+      <c r="S154" s="15" t="n">
         <v>0.0299</v>
       </c>
-      <c r="T154" s="16" t="n">
+      <c r="T154" s="15" t="n">
         <v>0.0023</v>
       </c>
       <c r="U154" s="0" t="n">
@@ -6137,10 +6112,10 @@
       <c r="R155" s="0" t="n">
         <v>30</v>
       </c>
-      <c r="S155" s="16" t="n">
+      <c r="S155" s="15" t="n">
         <v>0.019</v>
       </c>
-      <c r="T155" s="16" t="n">
+      <c r="T155" s="15" t="n">
         <v>0.004</v>
       </c>
       <c r="U155" s="0" t="n">

</xml_diff>